<commit_message>
Cotações atualizadas - 2026-09-05
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E360"/>
+  <dimension ref="A1:E361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9434,6 +9434,31 @@
         </is>
       </c>
     </row>
+    <row r="361">
+      <c r="A361" s="2" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>26,3905</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>19,2756</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>17,3452</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>17,3452</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-06
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E361"/>
+  <dimension ref="A1:E362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9459,6 +9459,31 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>26,3905</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>19,2756</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>17,3452</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>17,3452</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-07
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E362"/>
+  <dimension ref="A1:E363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9484,6 +9484,31 @@
         </is>
       </c>
     </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>26,4251</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>19,2096</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>17,3812</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>17,3812</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-08
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E363"/>
+  <dimension ref="A1:E364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9509,6 +9509,31 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>26,3945</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>19,2148</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>19,2148</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>19,2148</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-09
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E364"/>
+  <dimension ref="A1:E365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9534,6 +9534,31 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>26,3573</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>19,1479</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>17,2825</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>17,2825</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-10
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E365"/>
+  <dimension ref="A1:E366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9559,6 +9559,31 @@
         </is>
       </c>
     </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>26,0246</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>18,9846</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>16,9915</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>16,9915</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-11
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E366"/>
+  <dimension ref="A1:E367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9584,6 +9584,31 @@
         </is>
       </c>
     </row>
+    <row r="367">
+      <c r="A367" s="2" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>26,0154</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>18,9095</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-12
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E367"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9609,6 +9609,31 @@
         </is>
       </c>
     </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>26,0154</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>18,9095</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-13
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9634,6 +9634,31 @@
         </is>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>26,0154</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>18,9095</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>16,8985</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-14
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:E370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9659,6 +9659,31 @@
         </is>
       </c>
     </row>
+    <row r="370">
+      <c r="A370" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>26,2222</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>19,1239</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>17,0191</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>17,0191</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-15
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E370"/>
+  <dimension ref="A1:E371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9684,6 +9684,31 @@
         </is>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>25,8886</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>19,1465</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>16,8827</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>16,8827</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-16
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E371"/>
+  <dimension ref="A1:E372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9709,6 +9709,31 @@
         </is>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" s="2" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>25,9527</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>19,0403</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>16,7925</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>16,7925</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-17
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E372"/>
+  <dimension ref="A1:E373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9734,6 +9734,31 @@
         </is>
       </c>
     </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>26,0884</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>12,4797</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>16,9118</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>16,9118</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-18
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9759,6 +9759,31 @@
         </is>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>26,3513</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>19,3391</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-19
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E374"/>
+  <dimension ref="A1:E375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9784,6 +9784,31 @@
         </is>
       </c>
     </row>
+    <row r="375">
+      <c r="A375" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>26,3513</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>19,3391</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-20
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E375"/>
+  <dimension ref="A1:E376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9809,6 +9809,31 @@
         </is>
       </c>
     </row>
+    <row r="376">
+      <c r="A376" s="2" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>26,3513</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>19,3391</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>17,0995</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-21
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E376"/>
+  <dimension ref="A1:E377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9834,6 +9834,31 @@
         </is>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>25,9214</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>19,2979</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>16,8953</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>16,8953</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-22
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E377"/>
+  <dimension ref="A1:E378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9859,6 +9859,31 @@
         </is>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" s="2" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>26,2093</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>19,6154</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>17,1233</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>17,1233</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-23
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E378"/>
+  <dimension ref="A1:E379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9884,6 +9884,31 @@
         </is>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" s="2" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>26,2093</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>19,6983</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>17,1304</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>17,1304</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-24
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E379"/>
+  <dimension ref="A1:E380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9909,6 +9909,31 @@
         </is>
       </c>
     </row>
+    <row r="380">
+      <c r="A380" s="2" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>26,1233</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>19,6175</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>17,0621</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>17,0621</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-25
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E380"/>
+  <dimension ref="A1:E381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9934,6 +9934,31 @@
         </is>
       </c>
     </row>
+    <row r="381">
+      <c r="A381" s="2" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>26,0506</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>19,5766</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-26
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E381"/>
+  <dimension ref="A1:E382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9959,6 +9959,31 @@
         </is>
       </c>
     </row>
+    <row r="382">
+      <c r="A382" s="2" t="n">
+        <v>46291</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>26,0506</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>19,5766</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-27
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E382"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9984,6 +9984,31 @@
         </is>
       </c>
     </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>26,0506</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>19,5766</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>17,0211</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-29
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10009,6 +10009,31 @@
         </is>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" s="2" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>26,1979</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>19,6467</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>17,1055</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>17,1055</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-09-30
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E384"/>
+  <dimension ref="A1:E385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10034,6 +10034,31 @@
         </is>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" s="2" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>26,0602</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>19,6397</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>17,1083</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>17,1083</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-01
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E385"/>
+  <dimension ref="A1:E386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10059,6 +10059,31 @@
         </is>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" s="2" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>17,1258</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>19,6556</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>17,1258</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>17,1258</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-02
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E386"/>
+  <dimension ref="A1:E387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10084,6 +10084,31 @@
         </is>
       </c>
     </row>
+    <row r="387">
+      <c r="A387" s="2" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>25,8355</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>19,7812</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>17,0241</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>17,0241</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-03
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E387"/>
+  <dimension ref="A1:E388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10109,6 +10109,31 @@
         </is>
       </c>
     </row>
+    <row r="388">
+      <c r="A388" s="2" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>25,3249</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>19,7739</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>17,0241</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>17,0241</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-04
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E388"/>
+  <dimension ref="A1:E389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10134,6 +10134,31 @@
         </is>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" s="2" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>25,3249</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>19,7739</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>16,9196</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>16,9196</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-06
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E389"/>
+  <dimension ref="A1:E390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10159,6 +10159,31 @@
         </is>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" s="2" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>25,3821</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>19,9423</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>16,9196</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>16,9196</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-07
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E390"/>
+  <dimension ref="A1:E391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10184,6 +10184,31 @@
         </is>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" s="2" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>25,3807</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>12,8408</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>16,9185</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>16,9185</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-08
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10209,6 +10209,31 @@
         </is>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" s="2" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>16,9542</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>13,0269</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>16,9542</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>16,9542</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-09
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E392"/>
+  <dimension ref="A1:E393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10234,6 +10234,31 @@
         </is>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" s="2" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>25,3998</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>13,0355</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>16,7788</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>16,7788</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-10
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E393"/>
+  <dimension ref="A1:E394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10259,6 +10259,31 @@
         </is>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" s="2" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>25,1975</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>12,9099</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-11
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E394"/>
+  <dimension ref="A1:E395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10284,6 +10284,31 @@
         </is>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" s="2" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>25,1975</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>12,9099</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-12
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E395"/>
+  <dimension ref="A1:E396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10309,6 +10309,31 @@
         </is>
       </c>
     </row>
+    <row r="396">
+      <c r="A396" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>25,1975</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>12,9099</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>16,6084</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-13
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E396"/>
+  <dimension ref="A1:E397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10334,6 +10334,31 @@
         </is>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" s="2" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>25,2932</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>12,8233</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>16,7623</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>16,7623</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-14
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E397"/>
+  <dimension ref="A1:E398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10359,6 +10359,31 @@
         </is>
       </c>
     </row>
+    <row r="398">
+      <c r="A398" s="2" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>16,8523</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>14,6636</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>16,8523</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>16,8523</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-15
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10384,6 +10384,31 @@
         </is>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" s="2" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>25,6437</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>12,7799</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>16,9082</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>16,9082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-16
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E399"/>
+  <dimension ref="A1:E400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10409,6 +10409,31 @@
         </is>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" s="2" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>25,6158</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>12,6426</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-17
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E400"/>
+  <dimension ref="A1:E401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10434,6 +10434,31 @@
         </is>
       </c>
     </row>
+    <row r="401">
+      <c r="A401" s="2" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>25,6158</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>12,6426</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-18
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E401"/>
+  <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10459,6 +10459,31 @@
         </is>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" s="2" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>25,6158</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>12,6426</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>16,9504</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-20
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10484,6 +10484,31 @@
         </is>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" s="2" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>25,8569</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>19,9823</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>17,0407</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>17,0407</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-21
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E403"/>
+  <dimension ref="A1:E404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10509,6 +10509,31 @@
         </is>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" s="2" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>25,5526</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>19,9777</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>16,8412</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>16,8412</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-22
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E404"/>
+  <dimension ref="A1:E405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10534,6 +10534,31 @@
         </is>
       </c>
     </row>
+    <row r="405">
+      <c r="A405" s="2" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>25,7765</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>12,5218</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>17,0214</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>17,0214</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-23
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E405"/>
+  <dimension ref="A1:E406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10559,6 +10559,31 @@
         </is>
       </c>
     </row>
+    <row r="406">
+      <c r="A406" s="2" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>25,2787</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>19,8157</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-24
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E406"/>
+  <dimension ref="A1:E407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10584,6 +10584,31 @@
         </is>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" s="2" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>25,2787</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>19,8157</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-25
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E407"/>
+  <dimension ref="A1:E408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10609,6 +10609,31 @@
         </is>
       </c>
     </row>
+    <row r="408">
+      <c r="A408" s="2" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>25,2787</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>19,8157</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>16,8025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-27
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E408"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10634,6 +10634,31 @@
         </is>
       </c>
     </row>
+    <row r="409">
+      <c r="A409" s="2" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>25,3165</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>19,8372</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>19,8372</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>19,8372</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-28
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:E410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10659,6 +10659,31 @@
         </is>
       </c>
     </row>
+    <row r="410">
+      <c r="A410" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>25,3339</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>19,9064</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>16,8268</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>16,8268</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-29
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E410"/>
+  <dimension ref="A1:E411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10684,6 +10684,31 @@
         </is>
       </c>
     </row>
+    <row r="411">
+      <c r="A411" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>20,1632</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>12,4716</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>12,4716</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>12,4716</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-30
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E411"/>
+  <dimension ref="A1:E412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10709,6 +10709,31 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>25,2109</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>12,5341</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>17,0176</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>17,0176</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cotações atualizadas - 2026-10-31
</commit_message>
<xml_diff>
--- a/cotacoes_fundos_cgd.xlsx
+++ b/cotacoes_fundos_cgd.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E412"/>
+  <dimension ref="A1:E413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10734,6 +10734,31 @@
         </is>
       </c>
     </row>
+    <row r="413">
+      <c r="A413" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>25,2498</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>12,5595</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>17,1304</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>17,1304</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>